<commit_message>
Update slab delivery cases and manual registry
</commit_message>
<xml_diff>
--- a/output/manual_values_registry.xlsx
+++ b/output/manual_values_registry.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,23 +25,13 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <sz val="10"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D9D9D9"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -56,9 +46,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -424,50 +413,50 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G31"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="46" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
-    <col hidden="1" width="22" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col hidden="1" width="20" customWidth="1" min="6" max="6"/>
     <col hidden="1" width="30" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Раздел</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Наименование</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Ед. изм.</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Типовое значение</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Комментарий</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>section_code</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>key</t>
         </is>
@@ -481,19 +470,15 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Доставка арматуры и металла, машины</t>
+          <t>Подача арматуры автокраном, смены</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>маш</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Не выделено отдельной строкой в смете АРК (раздел проверен) — оставлено пустым.</t>
-        </is>
-      </c>
+          <t>смена</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
           <t>foundation_slab</t>
@@ -501,7 +486,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>rebar_metal_delivery_trucks</t>
+          <t>rebar_crane_shifts</t>
         </is>
       </c>
     </row>
@@ -513,17 +498,20 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Общий вес металла коробки для контроля доставки</t>
+          <t>Работа бетононасоса, смены</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>кг</t>
-        </is>
+          <t>смена</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>1</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Не выделено отдельной строкой в смете АРК (раздел проверен) — оставлено пустым. Контрольное поле коробки поставки, не строка сметы.</t>
+          <t>Из сметы АРК: «Работа бетононасоса 36м», раздел «Устройство фундаментной плиты», 1 смена.</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -533,7 +521,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>box_total_metal_weight_kg</t>
+          <t>concrete_pump_shifts</t>
         </is>
       </c>
     </row>
@@ -545,20 +533,20 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Работа бетононасоса, смены</t>
+          <t>Логистика и снабжение</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>смена</t>
+          <t>руб</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1</v>
+        <v>26180</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Из сметы АРК: «Работа бетононасоса 36м», раздел «Устройство фундаментной плиты», 1 смена.</t>
+          <t>Из сметы АРК: «Логистика, и снабжение», раздел «Устройство фундаментной плиты», 26180 руб. Сумма в рублях из сметы АРК — масштабируется под объём/бюджет проекта, не универсальная константа; проверяйте перед использованием на другом проекте.</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -568,7 +556,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>concrete_pump_shifts</t>
+          <t>logistics_and_supply_amount</t>
         </is>
       </c>
     </row>
@@ -580,7 +568,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Логистика и снабжение</t>
+          <t>Расходные материалы, амортизация инструмента</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -589,11 +577,11 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>26180</v>
+        <v>52361</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Из сметы АРК: «Логистика, и снабжение», раздел «Устройство фундаментной плиты», 26180 руб. Сумма в рублях из сметы АРК — масштабируется под объём/бюджет проекта, не универсальная константа; проверяйте перед использованием на другом проекте.</t>
+          <t>Из сметы АРК: «Расходные материалы, амортизация инструмента», тот же раздел, 52361 руб. Сумма в рублях из сметы АРК — масштабируется под объём/бюджет проекта, не универсальная константа; проверяйте перед использованием на другом проекте.</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -603,42 +591,39 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>logistics_and_supply_amount</t>
+          <t>consumables_tool_amortization_amount</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Фундаментная плита</t>
+          <t>Стены и перемычки</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Расходные материалы, амортизация инструмента</t>
+          <t>Доставка бетона до объекта, рейсов, 2-й этаж</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>руб</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>52361</v>
+          <t>рейс</t>
+        </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Из сметы АРК: «Расходные материалы, амортизация инструмента», тот же раздел, 52361 руб. Сумма в рублях из сметы АРК — масштабируется под объём/бюджет проекта, не универсальная константа; проверяйте перед использованием на другом проекте.</t>
+          <t>Не выделено отдельной строкой в смете АРК (раздел проверен) — оставлено пустым. Для надстройки 2 света отдельной доставки бетона под перемычки в смете нет.</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>foundation_slab</t>
+          <t>load_bearing_walls_lintels</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>consumables_tool_amortization_amount</t>
+          <t>floor_2_concrete_delivery_trips</t>
         </is>
       </c>
     </row>
@@ -650,17 +635,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Доставка бетона до объекта, рейсов, 2-й этаж</t>
+          <t>Есть плоская кровля для парапета/вентканалов</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>рейс</t>
+          <t>да/нет</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Не выделено отдельной строкой в смете АРК (раздел проверен) — оставлено пустым. Для надстройки 2 света отдельной доставки бетона под перемычки в смете нет.</t>
+          <t>Проектно-зависимое булево поле (есть ли плоская кровля у парапета/вентканалов) — не подходит для общего справочника типовых значений, зависит от архитектуры конкретного проекта.</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -670,7 +655,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>floor_2_concrete_delivery_trips</t>
+          <t>flat_roof_enabled</t>
         </is>
       </c>
     </row>
@@ -682,17 +667,20 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Есть плоская кровля для парапета/вентканалов</t>
+          <t>Доставка бетона для перемычек, рейсы</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>да/нет</t>
-        </is>
+          <t>рейс</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>1</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Проектно-зависимое булево поле (есть ли плоская кровля у парапета/вентканалов) — не подходит для общего справочника типовых значений, зависит от архитектуры конкретного проекта.</t>
+          <t>Из сметы АРК: «Доставка бетона до объекта» сразу после бетонирования монолитных перемычек, 1-й этаж, 1 рейс.</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -702,7 +690,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>flat_roof_enabled</t>
+          <t>concrete_delivery_trips</t>
         </is>
       </c>
     </row>
@@ -714,12 +702,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Доставка бетона для перемычек, рейсы</t>
+          <t>Кран для парапета, смены</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>рейс</t>
+          <t>смена</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -727,7 +715,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Из сметы АРК: «Доставка бетона до объекта» сразу после бетонирования монолитных перемычек, 1-й этаж, 1 рейс.</t>
+          <t>Из сметы АРК: «Перемещение блоков, смеси автокраном», раздел «Парапеты», 1 смена.</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -737,7 +725,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>concrete_delivery_trips</t>
+          <t>parapet_crane_shifts</t>
         </is>
       </c>
     </row>
@@ -749,20 +737,20 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Кран для парапета, смены</t>
+          <t>Вывоз мусора, машины</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>смена</t>
+          <t>маш</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Из сметы АРК: «Перемещение блоков, смеси автокраном», раздел «Парапеты», 1 смена.</t>
+          <t>Из сметы АРК: «Вывоз мусора с объекта», раздел стен/парапетов, 3 машины.</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -772,7 +760,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>parapet_crane_shifts</t>
+          <t>waste_removal_trucks</t>
         </is>
       </c>
     </row>
@@ -784,20 +772,20 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Вывоз мусора, машины</t>
+          <t>Расходные материалы и амортизация инструмента</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>маш</t>
+          <t>руб.</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>3</v>
+        <v>51577</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Из сметы АРК: «Вывоз мусора с объекта», раздел стен/парапетов, 3 машины.</t>
+          <t>Из сметы АРК: «Расходные материалы, амортизация инструмента», раздел «Парапеты», 51577 руб. Сумма в рублях из сметы АРК — масштабируется под объём/бюджет проекта, не универсальная константа; проверяйте перед использованием на другом проекте.</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -807,42 +795,35 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>waste_removal_trucks</t>
+          <t>walls_consumables_tool_amortization_amount_raw</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Стены и перемычки</t>
+          <t>Перекрытие 1 этажа</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Расходные материалы и амортизация инструмента</t>
+          <t>Подача опалубки и арматуры краном</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>руб.</t>
-        </is>
-      </c>
-      <c r="D12" t="n">
-        <v>51577</v>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Из сметы АРК: «Расходные материалы, амортизация инструмента», раздел «Парапеты», 51577 руб. Сумма в рублях из сметы АРК — масштабируется под объём/бюджет проекта, не универсальная константа; проверяйте перед использованием на другом проекте.</t>
-        </is>
-      </c>
+          <t>смена</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
-          <t>load_bearing_walls_lintels</t>
+          <t>floor_slab_1</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>walls_consumables_tool_amortization_amount_raw</t>
+          <t>formwork_rebar_crane_shifts</t>
         </is>
       </c>
     </row>
@@ -953,7 +934,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Работа бетононасоса</t>
+          <t>Подача опалубки и арматуры краном</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -961,14 +942,7 @@
           <t>смена</t>
         </is>
       </c>
-      <c r="D16" t="n">
-        <v>1</v>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>Из сметы АРК: «Работа бетононасоса 40м», плита перекрытия на отм.+4.980, 1 смена.</t>
-        </is>
-      </c>
+      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
           <t>floor_slab_2</t>
@@ -976,35 +950,42 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>concrete_pump_shifts</t>
+          <t>crane_shifts</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Кровля</t>
+          <t>Перекрытие 2 этажа</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Коэффициент работ кровли</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr"/>
+          <t>Работа бетононасоса</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>смена</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>1</v>
+      </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Не выделено отдельной строкой в смете АРК (раздел проверен) — оставлено пустым. Внутренний коэффициент калькулятора, не отдельная строка сметы.</t>
+          <t>Из сметы АРК: «Работа бетононасоса 40м», плита перекрытия на отм.+4.980, 1 смена.</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>flat_roof</t>
+          <t>floor_slab_2</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>roof_work_coeff</t>
+          <t>concrete_pump_shifts</t>
         </is>
       </c>
     </row>
@@ -1016,20 +997,13 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>ЭППС 50 мм, требуемый объем поставщика</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>м3</t>
-        </is>
-      </c>
-      <c r="D18" t="n">
-        <v>16.97312</v>
-      </c>
+          <t>Коэффициент работ кровли</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Из сметы АРК: «Утеплитель ЭППС ТЕХНОНИКОЛЬ CARBON PROF (50мм)», 16.97312 м3.</t>
+          <t>Не выделено отдельной строкой в смете АРК (раздел проверен) — оставлено пустым. Внутренний коэффициент калькулятора, не отдельная строка сметы.</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1039,7 +1013,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>eps50_supplier_required_volume_m3</t>
+          <t>roof_work_coeff</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1025,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>SLOPE плиты A, требуемый объем поставщика</t>
+          <t>ЭППС 50 мм, требуемый объем поставщика</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1060,11 +1034,11 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>5.2488</v>
+        <v>16.97312</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Из сметы АРК: SLOPE плиты A, уклон 2,1%, 5.2488 м3.</t>
+          <t>Из сметы АРК: «Утеплитель ЭППС ТЕХНОНИКОЛЬ CARBON PROF (50мм)», 16.97312 м3.</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1074,7 +1048,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>slope_plate_a_supplier_required_volume_m3</t>
+          <t>eps50_supplier_required_volume_m3</t>
         </is>
       </c>
     </row>
@@ -1086,7 +1060,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>SLOPE плиты B, требуемый объем поставщика</t>
+          <t>SLOPE плиты A, требуемый объем поставщика</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1095,11 +1069,11 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>9.576000000000001</v>
+        <v>5.2488</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Из сметы АРК: SLOPE плиты B, уклон 2,1%, 9.576 м3.</t>
+          <t>Из сметы АРК: SLOPE плиты A, уклон 2,1%, 5.2488 м3.</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1109,7 +1083,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>slope_plate_b_supplier_required_volume_m3</t>
+          <t>slope_plate_a_supplier_required_volume_m3</t>
         </is>
       </c>
     </row>
@@ -1121,7 +1095,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>SLOPE плиты J, требуемый объем поставщика</t>
+          <t>SLOPE плиты B, требуемый объем поставщика</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1130,11 +1104,11 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>1.7496</v>
+        <v>9.576000000000001</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Из сметы АРК: SLOPE плиты J, уклон 4,2%, 1.7496 м3.</t>
+          <t>Из сметы АРК: SLOPE плиты B, уклон 2,1%, 9.576 м3.</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1144,7 +1118,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>slope_plate_j_supplier_required_volume_m3</t>
+          <t>slope_plate_b_supplier_required_volume_m3</t>
         </is>
       </c>
     </row>
@@ -1156,7 +1130,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>SLOPE плиты K, требуемый объем поставщика</t>
+          <t>SLOPE плиты J, требуемый объем поставщика</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1165,11 +1139,11 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>1.9152</v>
+        <v>1.7496</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Из сметы АРК: SLOPE плиты K, уклон 4,2%, 1.9152 м3.</t>
+          <t>Из сметы АРК: SLOPE плиты J, уклон 4,2%, 1.7496 м3.</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1179,7 +1153,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>slope_plate_k_supplier_required_volume_m3</t>
+          <t>slope_plate_j_supplier_required_volume_m3</t>
         </is>
       </c>
     </row>
@@ -1191,17 +1165,20 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Примыкания к вентшахтам, количество</t>
+          <t>SLOPE плиты K, требуемый объем поставщика</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>шт</t>
-        </is>
+          <t>м3</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>1.9152</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Не выделено отдельной строкой в смете АРК (раздел проверен) — оставлено пустым. Длина примыканий в смете дана суммарно по мембране (не по количеству вентшахт отдельно).</t>
+          <t>Из сметы АРК: SLOPE плиты K, уклон 4,2%, 1.9152 м3.</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1211,7 +1188,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>vent_shaft_abutment_count</t>
+          <t>slope_plate_k_supplier_required_volume_m3</t>
         </is>
       </c>
     </row>
@@ -1223,7 +1200,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Отверстия в стенах из газоблока</t>
+          <t>Примыкания к вентшахтам, количество</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1233,7 +1210,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Не выделено отдельной строкой в смете АРК (раздел проверен) — оставлено пустым. В смете АРК воронки прямо указаны «без пробивки отверстий» — для этого проекта работа не заказывалась отдельно.</t>
+          <t>Не выделено отдельной строкой в смете АРК (раздел проверен) — оставлено пустым. Длина примыканий в смете дана суммарно по мембране (не по количеству вентшахт отдельно).</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1243,7 +1220,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>gas_block_wall_holes_count</t>
+          <t>vent_shaft_abutment_count</t>
         </is>
       </c>
     </row>
@@ -1255,20 +1232,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Подъем материалов автокраном</t>
+          <t>Отверстия в стенах из газоблока</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>смена</t>
-        </is>
-      </c>
-      <c r="D25" t="n">
-        <v>1</v>
+          <t>шт</t>
+        </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Из сметы АРК: «Подъем материалов автокраном», раздел «Кровельное покрытие», 1 смена.</t>
+          <t>Не выделено отдельной строкой в смете АРК (раздел проверен) — оставлено пустым. В смете АРК воронки прямо указаны «без пробивки отверстий» — для этого проекта работа не заказывалась отдельно.</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1278,7 +1252,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>roof_crane_lifting_shifts</t>
+          <t>gas_block_wall_holes_count</t>
         </is>
       </c>
     </row>
@@ -1290,20 +1264,20 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Расходные материалы кровли</t>
+          <t>Подъем материалов автокраном</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>руб.</t>
+          <t>смена</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>82101</v>
+        <v>1</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Из сметы АРК: «Расходные материалы, амортизация инструмента», раздел «Кровельное покрытие», 82101 руб. Сумма в рублях из сметы АРК — масштабируется под объём/бюджет проекта, не универсальная константа; проверяйте перед использованием на другом проекте.</t>
+          <t>Из сметы АРК: «Подъем материалов автокраном», раздел «Кровельное покрытие», 1 смена.</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1313,7 +1287,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>roof_consumables_total_raw</t>
+          <t>roof_crane_lifting_shifts</t>
         </is>
       </c>
     </row>
@@ -1325,20 +1299,20 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Вывоз мусора кровли</t>
+          <t>Расходные материалы кровли</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>маш</t>
+          <t>руб.</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>3</v>
+        <v>82101</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Из сметы АРК: «Вывоз мусора с объекта», раздел «Кровельное покрытие», 3 машины.</t>
+          <t>Из сметы АРК: «Расходные материалы, амортизация инструмента», раздел «Кровельное покрытие», 82101 руб. Сумма в рублях из сметы АРК — масштабируется под объём/бюджет проекта, не универсальная константа; проверяйте перед использованием на другом проекте.</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1348,7 +1322,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>roof_waste_removal_trucks</t>
+          <t>roof_consumables_total_raw</t>
         </is>
       </c>
     </row>
@@ -1360,20 +1334,20 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Логистика и снабжение кровли</t>
+          <t>Вывоз мусора кровли</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>руб.</t>
+          <t>маш</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>54734</v>
+        <v>3</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Из сметы АРК: «Логистика, и снабжение», раздел «Кровельное покрытие», 54734 руб. Сумма в рублях из сметы АРК — масштабируется под объём/бюджет проекта, не универсальная константа; проверяйте перед использованием на другом проекте.</t>
+          <t>Из сметы АРК: «Вывоз мусора с объекта», раздел «Кровельное покрытие», 3 машины.</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1383,7 +1357,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>roof_logistics_and_supply_total_raw</t>
+          <t>roof_waste_removal_trucks</t>
         </is>
       </c>
     </row>
@@ -1395,7 +1369,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Технический надзор кровли</t>
+          <t>Логистика и снабжение кровли</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1404,11 +1378,11 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>12586</v>
+        <v>54734</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Из сметы АРК: «Технический надзор», раздел «Кровельное покрытие», 12586 руб. Сумма в рублях из сметы АРК — масштабируется под объём/бюджет проекта, не универсальная константа; проверяйте перед использованием на другом проекте.</t>
+          <t>Из сметы АРК: «Логистика, и снабжение», раздел «Кровельное покрытие», 54734 руб. Сумма в рублях из сметы АРК — масштабируется под объём/бюджет проекта, не универсальная константа; проверяйте перед использованием на другом проекте.</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1418,7 +1392,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>technical_supervision_work_total</t>
+          <t>roof_logistics_and_supply_total_raw</t>
         </is>
       </c>
     </row>
@@ -1430,7 +1404,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Заготовительно-складские расходы кровли</t>
+          <t>Технический надзор кровли</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1439,11 +1413,11 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>58582</v>
+        <v>12586</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Из сметы АРК: «Заготовительно-складские расходы», раздел «Кровельное покрытие», 58582 руб. Сумма в рублях из сметы АРК — масштабируется под объём/бюджет проекта, не универсальная константа; проверяйте перед использованием на другом проекте.</t>
+          <t>Из сметы АРК: «Технический надзор», раздел «Кровельное покрытие», 12586 руб. Сумма в рублях из сметы АРК — масштабируется под объём/бюджет проекта, не универсальная константа; проверяйте перед использованием на другом проекте.</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1453,40 +1427,75 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>procurement_storage_work_total</t>
+          <t>technical_supervision_work_total</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Вентканалы Schiedel</t>
+          <t>Кровля</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
+          <t>Заготовительно-складские расходы кровли</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>руб.</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>58582</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Из сметы АРК: «Заготовительно-складские расходы», раздел «Кровельное покрытие», 58582 руб. Сумма в рублях из сметы АРК — масштабируется под объём/бюджет проекта, не универсальная константа; проверяйте перед использованием на другом проекте.</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>flat_roof</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>procurement_storage_work_total</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Вентиляционные каналы Schiedel</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
           <t>Количество доставок вентканалов</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C32" t="inlineStr">
         <is>
           <t>маш</t>
         </is>
       </c>
-      <c r="D31" t="n">
+      <c r="D32" t="n">
         <v>1</v>
       </c>
-      <c r="E31" t="inlineStr">
+      <c r="E32" t="inlineStr">
         <is>
           <t>Из сметы АРК: «Доставка вентканалов», раздел «Вентиляционные каналы Schiedel», 1 машина.</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr">
+      <c r="F32" t="inlineStr">
         <is>
           <t>schiedel_vent_channels</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr">
+      <c r="G32" t="inlineStr">
         <is>
           <t>schiedel_delivery_trips</t>
         </is>

</xml_diff>

<commit_message>
Refine review workbook manual controls
</commit_message>
<xml_diff>
--- a/output/manual_values_registry.xlsx
+++ b/output/manual_values_registry.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -506,14 +506,7 @@
           <t>смена</t>
         </is>
       </c>
-      <c r="D3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Из сметы АРК: «Работа бетононасоса 36м», раздел «Устройство фундаментной плиты», 1 смена.</t>
-        </is>
-      </c>
+      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
           <t>foundation_slab</t>
@@ -528,70 +521,56 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Фундаментная плита</t>
+          <t>Стены и перемычки</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Логистика и снабжение</t>
+          <t>Доставка бетона до объекта, рейсов, 2-й этаж</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>руб</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>26180</v>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Из сметы АРК: «Логистика, и снабжение», раздел «Устройство фундаментной плиты», 26180 руб. Сумма в рублях из сметы АРК — масштабируется под объём/бюджет проекта, не универсальная константа; проверяйте перед использованием на другом проекте.</t>
-        </is>
-      </c>
+          <t>рейс</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>foundation_slab</t>
+          <t>load_bearing_walls_lintels</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>logistics_and_supply_amount</t>
+          <t>floor_2_concrete_delivery_trips</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Фундаментная плита</t>
+          <t>Стены и перемычки</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Расходные материалы, амортизация инструмента</t>
+          <t>Есть плоская кровля для парапета/вентканалов</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>руб</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>52361</v>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Из сметы АРК: «Расходные материалы, амортизация инструмента», тот же раздел, 52361 руб. Сумма в рублях из сметы АРК — масштабируется под объём/бюджет проекта, не универсальная константа; проверяйте перед использованием на другом проекте.</t>
-        </is>
-      </c>
+          <t>да/нет</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
-          <t>foundation_slab</t>
+          <t>load_bearing_walls_lintels</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>consumables_tool_amortization_amount</t>
+          <t>flat_roof_enabled</t>
         </is>
       </c>
     </row>
@@ -603,7 +582,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Доставка бетона до объекта, рейсов, 2-й этаж</t>
+          <t>Доставка бетона для перемычек, рейсы</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -611,11 +590,7 @@
           <t>рейс</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Не выделено отдельной строкой в смете АРК (раздел проверен) — оставлено пустым. Для надстройки 2 света отдельной доставки бетона под перемычки в смете нет.</t>
-        </is>
-      </c>
+      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
           <t>load_bearing_walls_lintels</t>
@@ -623,7 +598,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>floor_2_concrete_delivery_trips</t>
+          <t>concrete_delivery_trips</t>
         </is>
       </c>
     </row>
@@ -635,19 +610,15 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Есть плоская кровля для парапета/вентканалов</t>
+          <t>Кран для парапета, смены</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>да/нет</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Проектно-зависимое булево поле (есть ли плоская кровля у парапета/вентканалов) — не подходит для общего справочника типовых значений, зависит от архитектуры конкретного проекта.</t>
-        </is>
-      </c>
+          <t>смена</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>load_bearing_walls_lintels</t>
@@ -655,7 +626,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>flat_roof_enabled</t>
+          <t>parapet_crane_shifts</t>
         </is>
       </c>
     </row>
@@ -667,22 +638,15 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Доставка бетона для перемычек, рейсы</t>
+          <t>Вывоз мусора, машины</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>рейс</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Из сметы АРК: «Доставка бетона до объекта» сразу после бетонирования монолитных перемычек, 1-й этаж, 1 рейс.</t>
-        </is>
-      </c>
+          <t>маш</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
           <t>load_bearing_walls_lintels</t>
@@ -690,19 +654,19 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>concrete_delivery_trips</t>
+          <t>waste_removal_trucks</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Стены и перемычки</t>
+          <t>Перекрытие 1 этажа</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Кран для парапета, смены</t>
+          <t>Подача опалубки и арматуры краном</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -710,132 +674,111 @@
           <t>смена</t>
         </is>
       </c>
-      <c r="D9" t="n">
-        <v>1</v>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Из сметы АРК: «Перемещение блоков, смеси автокраном», раздел «Парапеты», 1 смена.</t>
-        </is>
-      </c>
+      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
-          <t>load_bearing_walls_lintels</t>
+          <t>floor_slab_1</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>parapet_crane_shifts</t>
+          <t>formwork_rebar_crane_shifts</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Стены и перемычки</t>
+          <t>Перекрытие 1 этажа</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Вывоз мусора, машины</t>
+          <t>Работа бетононасоса</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>маш</t>
-        </is>
-      </c>
-      <c r="D10" t="n">
-        <v>3</v>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Из сметы АРК: «Вывоз мусора с объекта», раздел стен/парапетов, 3 машины.</t>
-        </is>
-      </c>
+          <t>смена</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
-          <t>load_bearing_walls_lintels</t>
+          <t>floor_slab_1</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>waste_removal_trucks</t>
+          <t>concrete_pump_shifts</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Стены и перемычки</t>
+          <t>Перекрытие 1 этажа</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Расходные материалы и амортизация инструмента</t>
+          <t>Эквивалент листов фанеры для свесов и доборов</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>руб.</t>
-        </is>
-      </c>
-      <c r="D11" t="n">
-        <v>51577</v>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>Из сметы АРК: «Расходные материалы, амортизация инструмента», раздел «Парапеты», 51577 руб. Сумма в рублях из сметы АРК — масштабируется под объём/бюджет проекта, не универсальная константа; проверяйте перед использованием на другом проекте.</t>
-        </is>
-      </c>
+          <t>лист</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
-          <t>load_bearing_walls_lintels</t>
+          <t>floor_slab_1</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>walls_consumables_tool_amortization_amount_raw</t>
+          <t>overhang_sheet_equivalent</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Перекрытие 1 этажа</t>
+          <t>Перекрытие 2 этажа</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Подача опалубки и арматуры краном</t>
+          <t>Коммерческое предложение поставщика на аренду опалубки, итого</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>смена</t>
+          <t>руб</t>
         </is>
       </c>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
-          <t>floor_slab_1</t>
+          <t>floor_slab_2</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>formwork_rebar_crane_shifts</t>
+          <t>formwork_rental_supplier_quote_total</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Перекрытие 1 этажа</t>
+          <t>Перекрытие 2 этажа</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Работа бетононасоса</t>
+          <t>Подача опалубки и арматуры краном</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -843,149 +786,123 @@
           <t>смена</t>
         </is>
       </c>
-      <c r="D13" t="n">
-        <v>1</v>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>Из сметы АРК: «Работа бетононасоса 40м», плита перекрытия на отм.+3.550, 1 смена.</t>
-        </is>
-      </c>
+      <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
-          <t>floor_slab_1</t>
+          <t>floor_slab_2</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>concrete_pump_shifts</t>
+          <t>crane_shifts</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Перекрытие 1 этажа</t>
+          <t>Перекрытие 2 этажа</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Эквивалент листов фанеры для свесов и доборов</t>
+          <t>Работа бетононасоса</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>лист</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>Не выделено отдельной строкой в смете АРК (раздел проверен) — оставлено пустым. Это внутренний коэффициент калькулятора (эквивалент листов фанеры для доборов), в смете нет отдельной строки для него — там просто общее количество листов фанеры на все нужды плиты.</t>
-        </is>
-      </c>
+          <t>смена</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
-          <t>floor_slab_1</t>
+          <t>floor_slab_2</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>overhang_sheet_equivalent</t>
+          <t>concrete_pump_shifts</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Перекрытие 2 этажа</t>
+          <t>Кровля</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Коммерческое предложение поставщика на аренду опалубки, итого</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>руб</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>Не выделено отдельной строкой в смете АРК (раздел проверен) — оставлено пустым. Это контрольное значение (коммерческое предложение поставщика), используется только для сверки соотношения, в смете отдельно не показывается — комплект опалубки в смете дан уже готовой строкой по м2.</t>
-        </is>
-      </c>
+          <t>Коэффициент работ кровли</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr"/>
+      <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
-          <t>floor_slab_2</t>
+          <t>flat_roof</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>formwork_rental_supplier_quote_total</t>
+          <t>roof_work_coeff</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Перекрытие 2 этажа</t>
+          <t>Кровля</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Подача опалубки и арматуры краном</t>
+          <t>ЭППС 50 мм, требуемый объем поставщика</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>смена</t>
+          <t>м3</t>
         </is>
       </c>
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
-          <t>floor_slab_2</t>
+          <t>flat_roof</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>crane_shifts</t>
+          <t>eps50_supplier_required_volume_m3</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Перекрытие 2 этажа</t>
+          <t>Кровля</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Работа бетононасоса</t>
+          <t>SLOPE плиты A, требуемый объем поставщика</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>смена</t>
-        </is>
-      </c>
-      <c r="D17" t="n">
-        <v>1</v>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>Из сметы АРК: «Работа бетононасоса 40м», плита перекрытия на отм.+4.980, 1 смена.</t>
-        </is>
-      </c>
+          <t>м3</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
-          <t>floor_slab_2</t>
+          <t>flat_roof</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>concrete_pump_shifts</t>
+          <t>slope_plate_a_supplier_required_volume_m3</t>
         </is>
       </c>
     </row>
@@ -997,15 +914,15 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Коэффициент работ кровли</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr"/>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>Не выделено отдельной строкой в смете АРК (раздел проверен) — оставлено пустым. Внутренний коэффициент калькулятора, не отдельная строка сметы.</t>
-        </is>
-      </c>
+          <t>SLOPE плиты B, требуемый объем поставщика</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>м3</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr">
         <is>
           <t>flat_roof</t>
@@ -1013,7 +930,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>roof_work_coeff</t>
+          <t>slope_plate_b_supplier_required_volume_m3</t>
         </is>
       </c>
     </row>
@@ -1025,7 +942,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>ЭППС 50 мм, требуемый объем поставщика</t>
+          <t>SLOPE плиты J, требуемый объем поставщика</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1033,14 +950,7 @@
           <t>м3</t>
         </is>
       </c>
-      <c r="D19" t="n">
-        <v>16.97312</v>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>Из сметы АРК: «Утеплитель ЭППС ТЕХНОНИКОЛЬ CARBON PROF (50мм)», 16.97312 м3.</t>
-        </is>
-      </c>
+      <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr">
         <is>
           <t>flat_roof</t>
@@ -1048,7 +958,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>eps50_supplier_required_volume_m3</t>
+          <t>slope_plate_j_supplier_required_volume_m3</t>
         </is>
       </c>
     </row>
@@ -1060,7 +970,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>SLOPE плиты A, требуемый объем поставщика</t>
+          <t>SLOPE плиты K, требуемый объем поставщика</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1068,14 +978,7 @@
           <t>м3</t>
         </is>
       </c>
-      <c r="D20" t="n">
-        <v>5.2488</v>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>Из сметы АРК: SLOPE плиты A, уклон 2,1%, 5.2488 м3.</t>
-        </is>
-      </c>
+      <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr">
         <is>
           <t>flat_roof</t>
@@ -1083,7 +986,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>slope_plate_a_supplier_required_volume_m3</t>
+          <t>slope_plate_k_supplier_required_volume_m3</t>
         </is>
       </c>
     </row>
@@ -1095,22 +998,15 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>SLOPE плиты B, требуемый объем поставщика</t>
+          <t>Примыкания к вентшахтам, количество</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>м3</t>
-        </is>
-      </c>
-      <c r="D21" t="n">
-        <v>9.576000000000001</v>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>Из сметы АРК: SLOPE плиты B, уклон 2,1%, 9.576 м3.</t>
-        </is>
-      </c>
+          <t>шт</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
           <t>flat_roof</t>
@@ -1118,7 +1014,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>slope_plate_b_supplier_required_volume_m3</t>
+          <t>vent_shaft_abutment_count</t>
         </is>
       </c>
     </row>
@@ -1130,22 +1026,15 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>SLOPE плиты J, требуемый объем поставщика</t>
+          <t>Отверстия в стенах из газоблока</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>м3</t>
-        </is>
-      </c>
-      <c r="D22" t="n">
-        <v>1.7496</v>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>Из сметы АРК: SLOPE плиты J, уклон 4,2%, 1.7496 м3.</t>
-        </is>
-      </c>
+          <t>шт</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr">
         <is>
           <t>flat_roof</t>
@@ -1153,7 +1042,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>slope_plate_j_supplier_required_volume_m3</t>
+          <t>gas_block_wall_holes_count</t>
         </is>
       </c>
     </row>
@@ -1165,22 +1054,15 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>SLOPE плиты K, требуемый объем поставщика</t>
+          <t>Подъем материалов автокраном</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>м3</t>
-        </is>
-      </c>
-      <c r="D23" t="n">
-        <v>1.9152</v>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>Из сметы АРК: SLOPE плиты K, уклон 4,2%, 1.9152 м3.</t>
-        </is>
-      </c>
+          <t>смена</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr">
         <is>
           <t>flat_roof</t>
@@ -1188,7 +1070,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>slope_plate_k_supplier_required_volume_m3</t>
+          <t>roof_crane_lifting_shifts</t>
         </is>
       </c>
     </row>
@@ -1200,19 +1082,15 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Примыкания к вентшахтам, количество</t>
+          <t>Вывоз мусора кровли</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>шт</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>Не выделено отдельной строкой в смете АРК (раздел проверен) — оставлено пустым. Длина примыканий в смете дана суммарно по мембране (не по количеству вентшахт отдельно).</t>
-        </is>
-      </c>
+          <t>маш</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr">
         <is>
           <t>flat_roof</t>
@@ -1220,282 +1098,33 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>vent_shaft_abutment_count</t>
+          <t>roof_waste_removal_trucks</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Кровля</t>
+          <t>Вентиляционные каналы Schiedel</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Отверстия в стенах из газоблока</t>
+          <t>Количество доставок вентканалов</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>шт</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>Не выделено отдельной строкой в смете АРК (раздел проверен) — оставлено пустым. В смете АРК воронки прямо указаны «без пробивки отверстий» — для этого проекта работа не заказывалась отдельно.</t>
-        </is>
-      </c>
+          <t>маш</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr">
         <is>
-          <t>flat_roof</t>
+          <t>schiedel_vent_channels</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
-        <is>
-          <t>gas_block_wall_holes_count</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Кровля</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Подъем материалов автокраном</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>смена</t>
-        </is>
-      </c>
-      <c r="D26" t="n">
-        <v>1</v>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>Из сметы АРК: «Подъем материалов автокраном», раздел «Кровельное покрытие», 1 смена.</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>flat_roof</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>roof_crane_lifting_shifts</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Кровля</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Расходные материалы кровли</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>руб.</t>
-        </is>
-      </c>
-      <c r="D27" t="n">
-        <v>82101</v>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>Из сметы АРК: «Расходные материалы, амортизация инструмента», раздел «Кровельное покрытие», 82101 руб. Сумма в рублях из сметы АРК — масштабируется под объём/бюджет проекта, не универсальная константа; проверяйте перед использованием на другом проекте.</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>flat_roof</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>roof_consumables_total_raw</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Кровля</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Вывоз мусора кровли</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>маш</t>
-        </is>
-      </c>
-      <c r="D28" t="n">
-        <v>3</v>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>Из сметы АРК: «Вывоз мусора с объекта», раздел «Кровельное покрытие», 3 машины.</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>flat_roof</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>roof_waste_removal_trucks</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>Кровля</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Логистика и снабжение кровли</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>руб.</t>
-        </is>
-      </c>
-      <c r="D29" t="n">
-        <v>54734</v>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>Из сметы АРК: «Логистика, и снабжение», раздел «Кровельное покрытие», 54734 руб. Сумма в рублях из сметы АРК — масштабируется под объём/бюджет проекта, не универсальная константа; проверяйте перед использованием на другом проекте.</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>flat_roof</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>roof_logistics_and_supply_total_raw</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>Кровля</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Технический надзор кровли</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>руб.</t>
-        </is>
-      </c>
-      <c r="D30" t="n">
-        <v>12586</v>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>Из сметы АРК: «Технический надзор», раздел «Кровельное покрытие», 12586 руб. Сумма в рублях из сметы АРК — масштабируется под объём/бюджет проекта, не универсальная константа; проверяйте перед использованием на другом проекте.</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>flat_roof</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>technical_supervision_work_total</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>Кровля</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>Заготовительно-складские расходы кровли</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>руб.</t>
-        </is>
-      </c>
-      <c r="D31" t="n">
-        <v>58582</v>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>Из сметы АРК: «Заготовительно-складские расходы», раздел «Кровельное покрытие», 58582 руб. Сумма в рублях из сметы АРК — масштабируется под объём/бюджет проекта, не универсальная константа; проверяйте перед использованием на другом проекте.</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>flat_roof</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>procurement_storage_work_total</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>Вентиляционные каналы Schiedel</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>Количество доставок вентканалов</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>маш</t>
-        </is>
-      </c>
-      <c r="D32" t="n">
-        <v>1</v>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>Из сметы АРК: «Доставка вентканалов», раздел «Вентиляционные каналы Schiedel», 1 машина.</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>schiedel_vent_channels</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr">
         <is>
           <t>schiedel_delivery_trips</t>
         </is>

</xml_diff>

<commit_message>
Clean manual review inputs for roof
</commit_message>
<xml_diff>
--- a/output/manual_values_registry.xlsx
+++ b/output/manual_values_registry.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -478,7 +478,6 @@
           <t>смена</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
           <t>foundation_slab</t>
@@ -506,7 +505,6 @@
           <t>смена</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
           <t>foundation_slab</t>
@@ -534,7 +532,6 @@
           <t>рейс</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
           <t>load_bearing_walls_lintels</t>
@@ -562,7 +559,6 @@
           <t>да/нет</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>load_bearing_walls_lintels</t>
@@ -590,7 +586,6 @@
           <t>рейс</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
           <t>load_bearing_walls_lintels</t>
@@ -618,7 +613,6 @@
           <t>смена</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>load_bearing_walls_lintels</t>
@@ -646,7 +640,6 @@
           <t>маш</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
           <t>load_bearing_walls_lintels</t>
@@ -674,7 +667,6 @@
           <t>смена</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
           <t>floor_slab_1</t>
@@ -702,7 +694,6 @@
           <t>смена</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
           <t>floor_slab_1</t>
@@ -730,7 +721,6 @@
           <t>лист</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
           <t>floor_slab_1</t>
@@ -758,7 +748,6 @@
           <t>руб</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
           <t>floor_slab_2</t>
@@ -786,7 +775,6 @@
           <t>смена</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
           <t>floor_slab_2</t>
@@ -814,7 +802,6 @@
           <t>смена</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
           <t>floor_slab_2</t>
@@ -837,8 +824,6 @@
           <t>Коэффициент работ кровли</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
           <t>flat_roof</t>
@@ -866,7 +851,6 @@
           <t>м3</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
           <t>flat_roof</t>
@@ -886,15 +870,14 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>SLOPE плиты A, требуемый объем поставщика</t>
+          <t>Подъем материалов автокраном</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>м3</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr"/>
+          <t>смена</t>
+        </is>
+      </c>
       <c r="F17" t="inlineStr">
         <is>
           <t>flat_roof</t>
@@ -902,7 +885,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>slope_plate_a_supplier_required_volume_m3</t>
+          <t>roof_crane_lifting_shifts</t>
         </is>
       </c>
     </row>
@@ -914,15 +897,14 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>SLOPE плиты B, требуемый объем поставщика</t>
+          <t>Вывоз мусора кровли</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>м3</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr"/>
+          <t>маш</t>
+        </is>
+      </c>
       <c r="F18" t="inlineStr">
         <is>
           <t>flat_roof</t>
@@ -930,201 +912,32 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>slope_plate_b_supplier_required_volume_m3</t>
+          <t>roof_waste_removal_trucks</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Кровля</t>
+          <t>Вентиляционные каналы Schiedel</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>SLOPE плиты J, требуемый объем поставщика</t>
+          <t>Количество доставок вентканалов</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>м3</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr"/>
+          <t>маш</t>
+        </is>
+      </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>flat_roof</t>
+          <t>schiedel_vent_channels</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
-        <is>
-          <t>slope_plate_j_supplier_required_volume_m3</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Кровля</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>SLOPE плиты K, требуемый объем поставщика</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>м3</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>flat_roof</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>slope_plate_k_supplier_required_volume_m3</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Кровля</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Примыкания к вентшахтам, количество</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>шт</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>flat_roof</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>vent_shaft_abutment_count</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Кровля</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Отверстия в стенах из газоблока</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>шт</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>flat_roof</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>gas_block_wall_holes_count</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Кровля</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Подъем материалов автокраном</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>смена</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>flat_roof</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>roof_crane_lifting_shifts</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Кровля</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Вывоз мусора кровли</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>маш</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>flat_roof</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>roof_waste_removal_trucks</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Вентиляционные каналы Schiedel</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Количество доставок вентканалов</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>маш</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr"/>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>schiedel_vent_channels</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
         <is>
           <t>schiedel_delivery_trips</t>
         </is>

</xml_diff>

<commit_message>
Expose geotextile laying overlap and refinement depth as editable
Both were silent hardcoded DEFAULT constants with no per-project
visibility. Checked real Excel formulas across TRC/ARK/USV smetas:
manual_refinement_depth_m varies 0.08-0.10m (ARK/USV=0.08, TRC=0.10);
the geotextile laying labor overlap varies 1.0-1.2x and isn't a stable
system rule (TRC=1.1, ARK=1.2, USV=none). Moved both to sheet 01-1
(SUPPLIER_INPUT) with sane defaults so Elena can override per project
instead of the value being invisible and unchangeable. New
geotextile_laying_overlap_coeff field added to the calculator (previously
this multiplier didn't exist at all for the labor line, only for
material purchase). 0 regressions on the full earthworks_calculator
suite (8/8 cases).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/manual_values_registry.xlsx
+++ b/output/manual_values_registry.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -478,7 +478,6 @@
           <t>смена</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
           <t>foundation_slab</t>
@@ -506,7 +505,6 @@
           <t>смена</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
           <t>foundation_slab</t>
@@ -534,7 +532,6 @@
           <t>рейс</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
           <t>load_bearing_walls_lintels</t>
@@ -562,7 +559,6 @@
           <t>рейс</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>load_bearing_walls_lintels</t>
@@ -590,7 +586,6 @@
           <t>смена</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
           <t>load_bearing_walls_lintels</t>
@@ -618,7 +613,6 @@
           <t>маш</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>load_bearing_walls_lintels</t>
@@ -646,7 +640,6 @@
           <t>смена</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
           <t>floor_slab_1</t>
@@ -674,7 +667,6 @@
           <t>смена</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
           <t>floor_slab_1</t>
@@ -702,7 +694,6 @@
           <t>смена</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
           <t>floor_slab_2</t>
@@ -730,7 +721,6 @@
           <t>смена</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
           <t>floor_slab_2</t>
@@ -758,7 +748,6 @@
           <t>смена</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
           <t>flat_roof</t>
@@ -786,7 +775,6 @@
           <t>маш</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
           <t>flat_roof</t>
@@ -814,7 +802,6 @@
           <t>маш</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
           <t>schiedel_vent_channels</t>
@@ -823,6 +810,76 @@
       <c r="G14" t="inlineStr">
         <is>
           <t>schiedel_delivery_trips</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Земляные работы</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Глубина ручной доработки дна котлована</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>м</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Экскаватор копает котлован полностью, вручную дорабатывают тонкий верхний слой перед укладкой геотекстиля/песка. 0.08 подтверждено в АРК и ЮСВ; ТРЦ - 0.1 (проверить у Елены при заполнении, если не уверена).</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>earthworks</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>manual_refinement_depth_m</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Земляные работы</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Коэффициент нахлеста геотекстиля в работе (укладка)</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>НЕ системная константа - в ТРЦ 1.1, в АРК 1.2, в ЮСВ вообще без надбавки (1.0). Зависит от формы котлована/числа углов. По умолчанию 1.0 (без надбавки); впишите реальное число для проекта, если знаете.</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>earthworks</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>geotextile_laying_overlap_coeff</t>
         </is>
       </c>
     </row>

</xml_diff>